<commit_message>
Trazabilidad de cada tecnica con la clase y guia del curso en ruta, matriz y plan
</commit_message>
<xml_diff>
--- a/entrega/Proyecto1_Caso3_Grupo5/Matriz_Casos_de_Prueba_Grupo5.xlsx
+++ b/entrega/Proyecto1_Caso3_Grupo5/Matriz_Casos_de_Prueba_Grupo5.xlsx
@@ -685,7 +685,7 @@
       </c>
       <c r="E2" s="6" t="inlineStr">
         <is>
-          <t>Partición de equivalencia</t>
+          <t>Partición de equivalencia (Clase 5 · guía G5)</t>
         </is>
       </c>
       <c r="F2" s="6" t="inlineStr">
@@ -735,7 +735,7 @@
       </c>
       <c r="E3" s="6" t="inlineStr">
         <is>
-          <t>Partición de equivalencia</t>
+          <t>Partición de equivalencia (Clase 5 · guía G5)</t>
         </is>
       </c>
       <c r="F3" s="6" t="inlineStr">
@@ -785,7 +785,7 @@
       </c>
       <c r="E4" s="6" t="inlineStr">
         <is>
-          <t>Partición de equivalencia</t>
+          <t>Partición de equivalencia (Clase 5 · guía G5)</t>
         </is>
       </c>
       <c r="F4" s="6" t="inlineStr">
@@ -834,7 +834,7 @@
       </c>
       <c r="E5" s="6" t="inlineStr">
         <is>
-          <t>Partición de equivalencia</t>
+          <t>Partición de equivalencia (Clase 5 · guía G5)</t>
         </is>
       </c>
       <c r="F5" s="6" t="inlineStr">
@@ -883,7 +883,7 @@
       </c>
       <c r="E6" s="6" t="inlineStr">
         <is>
-          <t>Partición de equivalencia</t>
+          <t>Partición de equivalencia (Clase 5 · guía G5)</t>
         </is>
       </c>
       <c r="F6" s="6" t="inlineStr">
@@ -933,7 +933,7 @@
       </c>
       <c r="E7" s="6" t="inlineStr">
         <is>
-          <t>Partición de equivalencia</t>
+          <t>Partición de equivalencia (Clase 5 · guía G5)</t>
         </is>
       </c>
       <c r="F7" s="6" t="inlineStr">
@@ -983,7 +983,7 @@
       </c>
       <c r="E8" s="6" t="inlineStr">
         <is>
-          <t>Partición de equivalencia y Análisis de valores límite</t>
+          <t>Partición de equivalencia y Análisis de valores límite (Clase 5 · guías G5 y G1)</t>
         </is>
       </c>
       <c r="F8" s="6" t="inlineStr">
@@ -1033,7 +1033,7 @@
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>Partición de equivalencia</t>
+          <t>Partición de equivalencia (Clase 5 · guía G5)</t>
         </is>
       </c>
       <c r="F9" s="6" t="inlineStr">
@@ -1083,7 +1083,7 @@
       </c>
       <c r="E10" s="6" t="inlineStr">
         <is>
-          <t>Tabla de decisión y Transición de estados</t>
+          <t>Tabla de decisión y Transición de estados (Clase 5 · guías G2 y G3)</t>
         </is>
       </c>
       <c r="F10" s="6" t="inlineStr">
@@ -1134,7 +1134,7 @@
       </c>
       <c r="E11" s="6" t="inlineStr">
         <is>
-          <t>Partición de equivalencia</t>
+          <t>Partición de equivalencia (Clase 5 · guía G5)</t>
         </is>
       </c>
       <c r="F11" s="6" t="inlineStr">
@@ -1185,7 +1185,7 @@
       </c>
       <c r="E12" s="6" t="inlineStr">
         <is>
-          <t>Prueba basada en casos de uso</t>
+          <t>Prueba basada en casos de uso (Clase 5 · guía G4)</t>
         </is>
       </c>
       <c r="F12" s="6" t="inlineStr">
@@ -1235,7 +1235,7 @@
       </c>
       <c r="E13" s="6" t="inlineStr">
         <is>
-          <t>Transición de estados</t>
+          <t>Transición de estados (Clase 5 · guía G3)</t>
         </is>
       </c>
       <c r="F13" s="6" t="inlineStr">
@@ -1285,7 +1285,7 @@
       </c>
       <c r="E14" s="6" t="inlineStr">
         <is>
-          <t>Tabla de decisión</t>
+          <t>Tabla de decisión (Clase 5 · guía G2)</t>
         </is>
       </c>
       <c r="F14" s="6" t="inlineStr">
@@ -1336,7 +1336,7 @@
       </c>
       <c r="E15" s="6" t="inlineStr">
         <is>
-          <t>Prueba basada en casos de uso</t>
+          <t>Prueba basada en casos de uso (Clase 5 · guía G4)</t>
         </is>
       </c>
       <c r="F15" s="6" t="inlineStr">
@@ -1385,7 +1385,7 @@
       </c>
       <c r="E16" s="6" t="inlineStr">
         <is>
-          <t>Transición de estados</t>
+          <t>Transición de estados (Clase 5 · guía G3)</t>
         </is>
       </c>
       <c r="F16" s="6" t="inlineStr">
@@ -1435,7 +1435,7 @@
       </c>
       <c r="E17" s="6" t="inlineStr">
         <is>
-          <t>Partición de equivalencia</t>
+          <t>Partición de equivalencia (Clase 5 · guía G5)</t>
         </is>
       </c>
       <c r="F17" s="6" t="inlineStr">
@@ -1484,7 +1484,7 @@
       </c>
       <c r="E18" s="6" t="inlineStr">
         <is>
-          <t>Medición de rendimiento con umbral (prueba no funcional; no corresponde a las cinco técnicas de caja negra del temario). El análisis de valores límite quedó diseñado sobre el umbral de 2 s, pero no se ejecutó como tal: no se controlaron 1999/2000/2001 ms como entradas.</t>
+          <t>Medición de rendimiento con umbral (prueba no funcional; no corresponde a las cinco técnicas de caja negra del temario). El análisis de valores límite quedó diseñado sobre el umbral de 2 s, pero no se ejecutó como tal: no se controlaron 1999/2000/2001 ms como entradas. (Clase 5 · guía G1)</t>
         </is>
       </c>
       <c r="F18" s="6" t="inlineStr">
@@ -1534,7 +1534,7 @@
       </c>
       <c r="E19" s="6" t="inlineStr">
         <is>
-          <t>Tabla de decisión</t>
+          <t>Tabla de decisión (Clase 5 · guía G2)</t>
         </is>
       </c>
       <c r="F19" s="6" t="inlineStr">

</xml_diff>